<commit_message>
Remove retired BEAM branding; fix outdated names; templates as references
Templates no longer carry "BEAM Builder Template Pack" footers, and brain
sources credit the template pack and Joshua Grech directly. Outdated
names are corrected: Victoria's Building and Plumbing Commission (not the
VBA), Before You Dig Australia (not Dial Before You Dig), NCC (not BCA),
a state-neutral WHS regulator on the incident report, and no 50% deposit
in the estimate quote terms. The defects guide now describes statutory
warranties accurately by state.

PDFs are generated from brain pages by tools/build_pdfs.py, so they can't
drift from the brain again. tools/describe_templates.py writes a Structure
outline into every document page, so documents can be produced in any
format or on the user's own letterhead; every skill says how.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/excel/Trade_Based_Estimate_Workbook.xlsx
+++ b/templates/excel/Trade_Based_Estimate_Workbook.xlsx
@@ -2605,7 +2605,7 @@
     <row r="26" ht="15" customHeight="1" s="37">
       <c r="A26" s="71" t="inlineStr">
         <is>
-          <t>2. Payment terms: As per contract or 50% deposit, balance on completion.</t>
+          <t>2. Payment terms: as per the contract. Any deposit will not exceed the legal limit for building work in your state.</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
     <row r="29" ht="15" customHeight="1" s="37">
       <c r="A29" s="71" t="inlineStr">
         <is>
-          <t>5. Work carried out per Australian Standards and BCA requirements.</t>
+          <t>5. Work carried out to the National Construction Code (NCC) and relevant Australian Standards.</t>
         </is>
       </c>
     </row>
@@ -2654,9 +2654,9 @@
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A34:E34"/>
     <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A29:E29"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="A7:E7"/>

</xml_diff>